<commit_message>
docs: mark rig clip 1 recorded; add accents-are-signal rule learned from it
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -676,7 +676,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="56" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
@@ -722,10 +722,22 @@
           <t>Metronome 120 in one earbud. Count "one two three four five six seven eight" — one number per click, normal teaching voice. Repeat the 1–8 round FOUR times without stopping (~20 seconds total). Say nothing else before, during, or after.</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr"/>
-      <c r="M4" s="6" t="inlineStr"/>
-      <c r="N4" s="6" t="inlineStr"/>
-      <c r="O4" s="7" t="inlineStr"/>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="N4" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-06 bounce. System: 122.2 BPM ✓, counts 8 ✓, but heard 4/4 — flat accents make 2/4 vs 4/4 inaudible. Optional take 2 with clear ONE-two accents.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="56" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -1970,7 +1982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2067,70 +2079,77 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="41" customHeight="1">
       <c r="B15" s="10" t="inlineStr">
         <is>
+          <t>•  DO let your natural musical accents live — the ONE-two of a march, the lilt of a waltz. Accents aren't label-leaking; they're the very thing the system must learn to hear (clip 1 taught us this: flat counting made 2/4 indistinguishable from 4/4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="10" t="inlineStr">
+        <is>
           <t>•  A recording went wrong? Don't delete — record again and write 'take 2' in Take notes.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="10" t="inlineStr"/>
-    </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Reading the sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>•  White cells are pre-filled suggestions: BPM and counts you're welcome to change — if you do, put the real values in the yellow Actual columns.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>•  Yellow cells are yours to fill in after each clip.</t>
+          <t>•  White cells are pre-filled suggestions: BPM and counts you're welcome to change — if you do, put the real values in the yellow Actual columns.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>•  Row 2 of the Recordings tab is a grayed-out example of a finished row.</t>
+          <t>•  Yellow cells are yours to fill in after each clip.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="B21" s="10" t="inlineStr">
         <is>
+          <t>•  Row 2 of the Recordings tab is a grayed-out example of a finished row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="B22" s="10" t="inlineStr">
+        <is>
           <t>•  ★ in the Pri column = the ten most valuable clips.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="B22" s="10" t="inlineStr"/>
-    </row>
     <row r="23" ht="15" customHeight="1">
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Files</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>•  Name each memo with the row's Filename if it's easy; otherwise just keep the memos in row order — the sheet is the source of truth.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>•  Name each memo with the row's Filename if it's easy; otherwise just keep the memos in row order — the sheet is the source of truth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>•  When done, send the memos plus this sheet (or a photo of it) back.</t>
         </is>

</xml_diff>

<commit_message>
feat: rig clip 2 (waltz, triplet-counted) — the fusion-precedence finding
Ben's natural waltz counting ('ONE-and-ah' through 8, click on numbers)
is ADR-006's equivalence case in the flesh. Gemini's index-keyed marker
path recovered 90.8 BPM at 92% confidence (all 32 numbers) and was
outvoted by the onset path reading the triplet syllables at 215.9 →
final 108/4-4/duple, wrong on all three. Second real case (after
frappé's 163-vs-74) where the marker path beats onsets and loses —
interpret_meter's onset-first precedence predates ADR-010's marker
quality and is now the obvious next eval-gated change. Counts 8/8 via
numeric regime (2/2 on rig clips); exercise honestly Unknown at 0%.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -739,7 +739,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="56" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
@@ -789,10 +789,22 @@
           <t>Metronome 90. Count a waltz combination exactly the way you naturally count one — in 3s, in 6s, or across 8 — your habit IS the data. Three or four rounds. Then write in 'Actual counts' precisely how you counted one phrase (e.g. "counted 1-2-3 4-2-3, phrase = 8 bars").</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr"/>
-      <c r="M5" s="6" t="inlineStr"/>
-      <c r="N5" s="6" t="inlineStr"/>
-      <c r="O5" s="7" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07. Counted 'ONE-and-ah' 1-8 ×4, click on numbers. System: counts 8 ✓; final tempo 108/4-4 ✗ BUT Gemini markers had 90.8 @ 92% and lost the fusion vote — key finding, see baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -1982,7 +1994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="B1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>

</xml_diff>

<commit_message>
feat: rig clip 4 (6/8, accented) — first compound meter recognized
Ben's ONE/FOUR accents made Gemini hear 6/8 (a first), while the same
expressive delivery poisoned the onset tempo: agogic long-short IOI
pairs at bar boundaries dragged the median to 84.7 against a confirmed
100 click (spoken median 96.3 — on the click). Third consecutive clip
where the marker path was the most truthful signal while under its
arbitration gate. Candidate next change: dominant-cluster IOI for onset
tempo instead of global median. Take 1 bounced silent and was discarded
before entering the benchmark.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -857,7 +857,7 @@
       <c r="N6" s="6" t="inlineStr"/>
       <c r="O6" s="7" t="inlineStr"/>
     </row>
-    <row r="7" ht="56" customHeight="1">
+    <row r="7" ht="58" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
@@ -907,10 +907,22 @@
           <t>Compound meter. Set the metronome to 100 and count the 6/8 bar as you would for class — "one two three four five six" or "ONE-and-a-TWO-and-a" — whichever is natural. Four rounds. Write EXACTLY what you spoke in 'Take notes' and confirm the phrase length in 'Actual counts'.</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="7" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07, take 2 (take 1 bounced silent). FIRST 6/8 recognized — accents worked. Onset tempo dragged to 84.7 by agogic bar-boundary gaps (spoke 96.3 on the 100 click); tempo row honestly red. Markers 96.3@51% under gate again.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="43" customHeight="1">
       <c r="A8" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 3 (4/4 control) — first fully green real-audio row
102.3 vs 104 (1.6%, 94% conf), 4/4, 8 counts, subdivision none — every
pinned field correct. As the control for clip 4: plain delivery lands
within 2% like clips 1-2, proving the 6/8 tempo miss was accent-induced
agogics, which pins the justification for a dominant-cluster IOI change
in rhythm.py (next eval-gated candidate).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -806,7 +806,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
@@ -852,10 +852,22 @@
           <t>Same as clip 1 but metronome 104: count 1–8 four times through, one number per click, nothing else on the recording.</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr"/>
-      <c r="M6" s="6" t="inlineStr"/>
-      <c r="N6" s="6" t="inlineStr"/>
-      <c r="O6" s="7" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07. FIRST ALL-GREEN ROW: 102.3 (1.6%), 4/4, 8 counts, none — all correct. Control confirms clip 4's tempo miss was accent-induced. Clean headroom this time.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 5 (step_names, 2/4) — sparse-marker tempo/count miss
First step_names rig clip. Metronome 120 confirmed, but some counts were
left silent by design (no word on every click). Pipeline read 77.8 BPM
(4/4, duple) and 16 counts — all wrong, honestly red.

Root cause visible in the trace: Gemini numbers every spoken word as a
consecutive beat with no notion of a skipped count, so sparse markers
read as a slower tempo and undercount the phrase. Distinct from clip 4's
accent-agogics miss — here the marker stream itself is sparse relative
to the beat grid, not just unevenly timed.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -936,7 +936,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="43" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
@@ -982,10 +982,22 @@
           <t>No numbers anywhere in this one. Mark a simple 8-count exercise with step names only — "tendu front, and close, brush through, and side…" — each key word landing on a click. Two or three times through.</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr"/>
-      <c r="M8" s="6" t="inlineStr"/>
-      <c r="N8" s="6" t="inlineStr"/>
-      <c r="O8" s="7" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07. Step names only, 4 rounds of 8; some counts left silent (no word every click) by design. Pipeline read 77.8 BPM / 4/4 / 16 counts — all wrong. Root cause: Gemini numbers every spoken word as a consecutive beat with no notion of skipped counts, so sparse markers read as slower tempo and fewer counts. New failure mode vs clip 4 (sparse markers, not just uneven timing).</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="43" customHeight="1">
       <c r="A9" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 6 (step_names waltz, 3/4) — band-coincidence tempo miss
Metronome 90 confirmed, word on nearly every count with downbeat stress.
Pipeline read 130.2 BPM (4/4) and 16 counts — all wrong.

New variant of clip 2's waltz-precedence finding (ADR-013): the onset
reading (130.2) happens to land inside the 70-140 beat band, so
band-aware arbitration never triggers, even though it's wrong. Meanwhile
Gemini only classified the downbeat-stressed word of each bar as
marker_type=beat (18 markers, 33.7 BPM, 57% confidence) — a near-bar-rate
reading that's both outside the band and just under the 60% confidence
gate. Neither signal path is simultaneously correctly-banded and
correct, so arbitration has nothing to grab onto.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -999,7 +999,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="43" customHeight="1">
+    <row r="9" ht="90" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
@@ -1049,10 +1049,22 @@
           <t>Step names only, waltz feel, metronome 90. An 8-count balancé-ish phrase marked in words ("down and lift, and sway, and carry…"), two or three times through. No numbers at all.</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
-      <c r="O9" s="7" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07. Step names, downbeat-stressed waltz, word on nearly every count. Pipeline read 130.2 BPM / 4/4 / 16 counts — all wrong. New variant of clip 2s waltz finding: onset (130.2) lands inside the 70-140 beat band so ADR-013 arbitration never engages, and Gemini only tagged the downbeat word of each bar as marker_type=beat (18 markers, 33.7 BPM, 57% confidence) -- near-bar-rate and just under the 60% arbitration gate. Neither signal path both correctly banded and correct.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 7 (step_names, 4/4 control) — tempo green, counts red
Metronome 104 confirmed, plie/tendu pattern in step names, mostly clean
with a stray eighth-note syllable or two and one blank beat.

Tempo lands within the 8% tolerance (111.9 vs 104, rel_err=0.076) —
first step_names clip to go green on tempo. Meter reads subdivision
duple instead of none, plausibly from the stray syllables. Structure
undercounts (16 vs true 8), the same pattern seen on clips 5-6.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1066,7 +1066,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="75" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
@@ -1112,10 +1112,22 @@
           <t>Step names only at 104 in 4/4 — a plié or tendu pattern, 8 counts, two or three times through, words on the beat, zero numbers.</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr"/>
-      <c r="M10" s="6" t="inlineStr"/>
-      <c r="N10" s="6" t="inlineStr"/>
-      <c r="O10" s="7" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O10" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07. Plie/tendu pattern, step names, mostly clean with a stray 8th-note syllable or two and one blank beat. Pipeline: 111.9 BPM (7.6% err, within 8% tolerance) - GREEN. Meter subdivision read duple vs true none (the stray syllables) - red. Counts 16 vs true 8 - same undercount pattern as clips 5-6.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="43" customHeight="1">
       <c r="A11" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 8 (step_names, 6/8) — meter recognition fails on sparse markers
Metronome 100 (eighth-note clicks) confirmed, "IN-and-[ah] OUT-and-[ah]"
pattern per bar with only 4 of 6 syllables spoken (the "ah"s silent) —
same silent-count pattern as clips 5-7, now inside a compound-meter bar.
Bar-to-bar spacing in the trace still sits close to the true 3.6s grid.

Pipeline read 134.6 BPM (raw onset 67.3 x2 multiplier), meter defaulted
to 4/4, and counts abstained — all wrong. Sibling to clip 4's finding
(first 6/8 recognized, but tempo dragged by accent agogics): here meter
recognition itself fails, plausibly because the sparse-marker pattern is
harder to read as compound meter than as simple meter.

Completes Part 1 of the capture checklist (clips 1-8, clean baseline).
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1129,7 +1129,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="43" customHeight="1">
+    <row r="11" ht="90" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>8</v>
       </c>
@@ -1175,10 +1175,22 @@
           <t>Step names only with the 6/8 swing at 100 — think pas de basque / skipping feel. One 6-count (or your natural) phrase, three times through. Confirm phrase length in 'Actual counts'.</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr"/>
-      <c r="M11" s="6" t="inlineStr"/>
-      <c r="N11" s="6" t="inlineStr"/>
-      <c r="O11" s="7" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07, take 2 (take 1 was the wrong exercise -- triplet-over-8, replaced after clarifying the 6/8 assignment in chat). IN-and-[ah] OUT-and-[ah] per bar, but only 4 of 6 syllables spoken (ahs silent), same silent-count pattern as clips 5-7. Bar-to-bar timing still close to the true 3.6s grid. Pipeline: 134.6 BPM (raw 67.3 x2), meter defaulted to 4/4, counts abstained (evidence disagreed) - all red. Sibling to clip 4s finding but meter recognition itself fails here.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: rig clip 9 (interrupted 4/4) — tempo/meter survive, counts abstain
Metronome 104 confirmed, clean round 1, ~5s in-tempo teaching interruption
around count 3 of round 2, then resumed plus one more clean round.

Tempo (99.7, 4.1% err) and meter (4/4) both green — the interruption
didn't perturb onset-based tracking at all. Counts abstained (evidence
disagreed), which is the honest answer: the interruption genuinely makes
"how many counts is this phrase" ambiguous. First Part 2 (known-killers)
clip.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1199,7 +1199,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="56" customHeight="1">
+    <row r="13" ht="75" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
@@ -1249,10 +1249,22 @@
           <t>Count 1–8 once cleanly. Midway through the SECOND round, stop and explain something for about five seconds exactly like in class ("really lengthen through that arm, don't grip the barre") — then pick the counting back up and finish, plus one more clean round. The interruption is the point.</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr"/>
-      <c r="M13" s="6" t="inlineStr"/>
-      <c r="N13" s="6" t="inlineStr"/>
-      <c r="O13" s="7" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07. Clean round 1, ~5s in-tempo teaching interruption around count 3 of round 2, then resumed plus one more clean round. Pipeline: tempo 99.7 (4.1% err) and meter 4/4 both GREEN -- interruption didnt break tempo/meter tracking at all. Counts abstained (evidence disagreed) -- the interruption split the phrase and the two count signals disagreed, arguably the honest answer.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="43" customHeight="1">
       <c r="A14" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 10 (step_names, interrupted 4/4) — dense markers hold tempo
Metronome 104 confirmed, step names with a word on every count (no
silent-count gaps, unlike clips 5-8), interruption mid-second-round.

Tempo lands at 104.8 (0.8% error) — tightest yet on an interruption
clip, confirming dense markers keep tempo tracking solid even through an
interruption. Meter subdivision reads duple vs true none. Counts reads
12 vs true 8 (clip 9's numbers sibling abstained here instead of
committing to a wrong number).
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1266,7 +1266,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="43" customHeight="1">
+    <row r="14" ht="75" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
@@ -1312,10 +1312,22 @@
           <t>Same interruption trick but marking with step names only: mark the phrase once, stop mid-second-time to coach for ~5 seconds, then resume marking to the end.</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr"/>
-      <c r="M14" s="6" t="inlineStr"/>
-      <c r="N14" s="6" t="inlineStr"/>
-      <c r="O14" s="7" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07. Step names, word on every count (no gaps), interruption mid-second-round. Pipeline: tempo 104.8 (0.8% err) - GREEN, tightest yet on an interruption clip; dense markers held through the interruption. Meter subdivision duple vs true none - red. Counts 12 vs true 8 - red (clip 9 abstained here instead of committing wrong).</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="43" customHeight="1">
       <c r="A15" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 11 (4/4 with prep) — all-green row, prep boundary correct
Metronome 104 confirmed, in-tempo prep "five, six, seven, eight" then 1-8
counted twice through, prep deliberately excluded from the phrase.

Tempo (0.1% err), meter, and counts (8, matching truth) all correct —
the prep-vs-phrase boundary was handled correctly. Second all-green rig
row after clip 3. Oddity noted but unscored: structure also reported 2
side(s) on a one-side exercise.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1329,7 +1329,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="43" customHeight="1">
+    <row r="15" ht="75" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
@@ -1375,10 +1375,22 @@
           <t>In tempo, give the preparation first — "five, six, seven, eight" — then count 1–8 twice through. 'Counts per phrase' stays 8: the prep is NOT part of the phrase (that boundary is what we're testing).</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr"/>
-      <c r="M15" s="6" t="inlineStr"/>
-      <c r="N15" s="6" t="inlineStr"/>
-      <c r="O15" s="7" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07. In-tempo prep (5,6,7,8) then 1-8 twice through, prep excluded from the phrase. Pipeline: tempo 103.9 (0.1% err), meter 4/4, subdivision none, counts 8 - ALL GREEN. Prep-vs-phrase boundary correctly excluded. Oddity: structure also reported 2 side(s) though this is one-side (not scored, not in expect block).</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="56" customHeight="1">
       <c r="A16" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 12 (half-tempo, 4/4) — purpose-built killer confirms x2 bug
Metronome 60 confirmed (Ben's "quick reminder" voice — an exercise he'd
run at 120, marked at genuinely half speed), 2 clean rounds of 8.

Raw onset tempo read 62.2 BPM at 100% coverage and CV=0.00 — essentially
exact — but the low-tempo x2 band-normalization heuristic doubled it to
124.4 (scorer's own failure_mode: metric_level_x2). Counts landed
correct. Cleanest instance yet of the multiplier bug already seen
misfiring on clips 6 and 8: the checklist's purpose-built half-tempo
probe found exactly what it was designed to find.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1392,7 +1392,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="56" customHeight="1">
+    <row r="16" ht="90" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
@@ -1442,10 +1442,22 @@
           <t>The quick-reminder voice. Pick an exercise you'd RUN at 120, set the metronome to 60, and mark it at that half speed the way you would when time is short. Metronome column already says 60 (what you speak); write "intended 120" in 'Take notes' (or your actual pair if you chose different numbers).</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr"/>
-      <c r="M16" s="6" t="inlineStr"/>
-      <c r="N16" s="6" t="inlineStr"/>
-      <c r="O16" s="7" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. Deliberately slow quick-reminder voice (intended 120, spoken at 60), 2 clean rounds of 8, no gaps. Pipeline: raw onset read 62.2 BPM at 100% coverage, CV=0.00 (near-perfect, essentially exact) but got doubled to 124.4 by the low-tempo x2 band-normalization heuristic (named failure_mode=metric_level_x2 in the scorer) - RED. Counts (8) correct. Cleanest case yet of the multiplier bug also seen on clips 6 and 8 - the checklists purpose-built half-tempo probe found exactly what it was designed to find.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="69" customHeight="1">
       <c r="A17" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 13 (long fast frappé, 2/4 @160) — mirror of ADR-014's finding
Metronome 160 confirmed, step names, 8 fast sets of 8 (64 counts) —
"the most valuable clip on this sheet."

Raw onset tempo read 161.8 BPM (1.1% error, 83% confidence, 100%
coverage, CV=0.05 — essentially exact) but got halved to 80.9 because it
sits just above the 140 band ceiling. Mirror image of clip 12's finding:
too-fast instead of too-slow, same normalize_tempo() band-snap defect
(ADR-014). Meter scored equivalent_reading (0.5 credit) via the existing
surface-equivalence logic while tempo scored flatly wrong — a live
example of the scoring inconsistency ADR-014 calls out as follow-on
work. Counts undercounted (32 vs true 64), tracking the halved tempo.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1459,7 +1459,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="69" customHeight="1">
+    <row r="17" ht="105" customHeight="1">
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
@@ -1509,10 +1509,22 @@
           <t>THE most valuable clip on this sheet. A long, fast, frappé-style combination — 32 to 64 counts — marked with step names at speed (metronome 160, or 80 if you prefer feeling it in twos: note which in 'Take notes'). Write the exact phrase length you used in 'Actual counts'. This is the shape the system currently cannot crack.</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="6" t="inlineStr"/>
-      <c r="O17" s="7" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="n">
+        <v>160</v>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. Fast frappe-style, step names, 8 fast sets of 8 (64 counts). Pipeline: raw onset 161.8 BPM at 83% conf/100% coverage/CV=0.05 - essentially exact (1.1% err) - but band-snap halved it to 80.9 (4/4 duple) because 161.8 sits just above the 140 ceiling. Mirror image of clip 12s finding (ADR-014): too-fast instead of too-slow, same defect. Meter got equivalent_reading partial credit (0.5) via existing surface equivalence logic; tempo scored flatly wrong - the exact scoring inconsistency ADR-014 flags as follow-on work. Counts 32 vs true 64.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 14 (sustained adagio, 4/4 @63) — legato breaks onset segmentation
Metronome 63 confirmed, sustained/connected step-name marking (long
vowels, no clear word-boundary gaps), 8-count phrase x4 rounds.

Tempo read 92.2 (46% error) — wrong, but a distinct failure mode from
clips 12/13's ADR-014 band-snap defect: 92.2 isn't a clean x2/x3 ratio
of 63, and it already sits inside 70-140 so normalize_tempo() never
touches it. Gemini found no beats at all. Local onset sections read
92/54/94 BPM with CV up to 0.36 (vs 0.00-0.07 on clipped/counted takes),
suggesting sustained legato delivery confuses onset segmentation itself,
not the band-normalization step. Counts abstained.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1526,7 +1526,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="105" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
@@ -1572,10 +1572,22 @@
           <t>Slow sustained adagio marking at 63 — long vowels, connected words ("développééé… aaand carry… fondu dooown…"). One 8-count phrase, twice through.</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr"/>
-      <c r="M18" s="6" t="inlineStr"/>
-      <c r="N18" s="6" t="inlineStr"/>
-      <c r="O18" s="7" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="N18" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. Slow sustained adagio, long vowels/connected words, 8-count phrase x4 rounds. Pipeline: tempo 92.2 (46% err) - RED, but NOT the ADR-014 band-snap defect (92.2 isnt a clean x2/x3 of 63, and it already sits inside 70-140). Gemini found no beats at all (fully abstained). Likely the sustained/legato delivery confuses onset word-boundary segmentation directly - local sections read 92/54/94 BPM with CV up to 0.36, vs CV 0.00-0.07 on clipped/counted takes. Counts abstained.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="56" customHeight="1">
       <c r="A19" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 15 (triplet subdivision, 4/4 @80) — all-green, ADR-013 confirmed
Metronome 80 confirmed, "ONE-and-a-TWO-and-a" triplet subdivision on
numbers, 2 rounds of 8 — the real-world counterpart to the tier-0
synthetic triplet case ADR-013 fixed.

Tempo (1.0% err), meter (4/4 triplet), and counts (8) all correct. The
marker-based tempo (80.8, 90% confidence) correctly outvoted the
syllable-level onset reading (186.9, outside the beat band) — exactly
the band-aware arbitration mechanism ADR-013 introduced, now confirmed
on real human speech. Third all-green rig row after clips 3 and 11.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1589,7 +1589,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="56" customHeight="1">
+    <row r="19" ht="90" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
@@ -1639,10 +1639,22 @@
           <t>Metronome 80. Count with triplet subdivision — "ONE-and-a-TWO-and-a-THREE-and-a…" — numbers on the clicks, the little syllables evenly between them. Two rounds of 8. (This subdivision is a known machine-breaker — keep it steady.)</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr"/>
-      <c r="M19" s="6" t="inlineStr"/>
-      <c r="N19" s="6" t="inlineStr"/>
-      <c r="O19" s="7" t="inlineStr"/>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. ONE-and-a-TWO-and-a triplet subdivision, numbers, 2 rounds of 8. Pipeline: tempo 80.8 (1.0% err), meter 4/4 triplet, counts 8 - ALL GREEN. Marker path (80.8, 90% conf, 16 beats) correctly outvoted the syllable-level onset (186.9, outside band) - real-world confirmation of ADR-013 band-aware arbitration on the exact clip type it was built to fix. Third all-green rig row (after clips 3, 11).</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="43" customHeight="1">
       <c r="A20" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 16 (duple subdivision, 4/4 @104) — all-green, duple sibling of 15
Metronome 104 confirmed, "ONE-and-TWO-and" eighth-note subdivision on
numbers, 2 rounds of 8 — duple sibling of clip 15's triplet case.

Tempo (1.1% err), meter (4/4 duple), and counts (8) all correct. Marker
path (102.9, 92% confidence) again outvoted the syllable-level onset
(216.3, well outside the beat band), confirming ADR-013's arbitration
holds for the simpler subdivision too. Fifth all-green rig row. Aside:
the separate raw SubdivisionResult (unused by scoring) misread this as
triplet — only the arbitrated coherent path feeds meter_triple.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1656,7 +1656,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="43" customHeight="1">
+    <row r="20" ht="90" customHeight="1">
       <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
@@ -1702,10 +1702,22 @@
           <t>Metronome 104. Count with eighth-note subdivision — "ONE-and-TWO-and-THREE-and…" — numbers on the clicks, "and" exactly halfway between. Two rounds of 8.</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr"/>
-      <c r="M20" s="6" t="inlineStr"/>
-      <c r="N20" s="6" t="inlineStr"/>
-      <c r="O20" s="7" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N20" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. ONE-and-TWO-and eighth-note (duple) subdivision, numbers, 2 rounds of 8. Pipeline: tempo 102.9 (1.1% err), meter 4/4 duple, counts 8 - ALL GREEN. Marker path (102.9, 92% conf) again outvoted the syllable-level onset (216.3). Aside: the separate raw SubdivisionResult misread triplet at 100% conf, but that path is unused by scoring - only the arbitrated coherent answer counts. Fifth all-green rig row (clips 3, 11, 15).</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: rig clip 17 (vocables, 4/4 @100) — green scoring, transcript hallucination
Metronome 100 confirmed, "da da DA da" style vocables with intentional
duple subdivision, 2 rounds of 8. First vocables clip.

Tempo (0.5% err), meter (4/4 duple), and counts (8) all correct — sixth
all-green rig row. But the underlying Whisper transcript is fabricated:
it reads as literal English number words ("one and two three four five
six seven eight") despite Ben confirming only non-lexical sounds were
spoken — almost certainly the ballet-vocabulary initial_prompt biasing
transcription toward plausible counting words. Word timing survived
intact so numeric scoring passed, but a downstream consumer surfacing
"what Whisper heard" would show a fabricated transcript. Distinct defect
from the tempo/meter findings tracked elsewhere in this corpus.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1726,7 +1726,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="56" customHeight="1">
+    <row r="22" ht="105" customHeight="1">
       <c r="A22" s="4" t="n">
         <v>17</v>
       </c>
@@ -1772,10 +1772,22 @@
           <t>Mark with sounds instead of words — "da da DA da… and da-da… TA" — however you naturally vocalize a phrase. Any meter is fine: the sheet suggests 4/4 at 100, but if you change it, correct the Meter/'Actual BPM' cells. 8-count phrase, three times through.</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr"/>
-      <c r="M22" s="6" t="inlineStr"/>
-      <c r="N22" s="6" t="inlineStr"/>
-      <c r="O22" s="7" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N22" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. Vocables ("da da DA da" style) with intentional duple subdivision, 2 rounds of 8. Pipeline: tempo 99.5 (0.5% err), meter 4/4 duple, counts 8 - ALL GREEN on the numbers. BUT: Whispers transcript hallucinated literal number-words (one and two three...) instead of the actual vocable sounds - almost certainly the ballet-vocabulary prompt biasing transcription. Timing survived so scoring passed, but the literal transcript is fabricated - a distinct hallucination defect worth its own investigation. Sixth all-green rig row.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="56" customHeight="1">
       <c r="A23" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 18 (four-x-8 combination, 4/4) — phrase-grouping miss
Metronome 104 confirmed, four rounds of 1-8 with different inflections,
meant as one 32-count combination rather than four separate 8-count
phrases — that distinction is the test.

Tempo (0.9% err) and meter both correct. Structure read 8 counts, not
32 — the system hears four cycles of eight with no signal that they
form a single longer phrase. Distinct from clips 5-8's sparse-marker
undercount: every count was spoken cleanly here, so this is a pure
phrase-boundary/grouping miss, not a marker-density one.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1789,7 +1789,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="56" customHeight="1">
+    <row r="23" ht="90" customHeight="1">
       <c r="A23" s="4" t="n">
         <v>18</v>
       </c>
@@ -1839,10 +1839,22 @@
           <t>Count FOUR rounds of 1-to-8 that together form ONE 32-count combination — think of it as one long exercise, four eights. 'Counts per phrase' is already set to 32, NOT 8: machines hear four cycles of eight, and whether they realize it's one phrase is exactly the test.</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr"/>
-      <c r="M23" s="6" t="inlineStr"/>
-      <c r="N23" s="6" t="inlineStr"/>
-      <c r="O23" s="7" t="inlineStr"/>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N23" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. Four rounds of 1-8, different inflections, meant as ONE 32-count combination. Pipeline: tempo 104.9 (0.9% err) and meter 4/4 both correct. Structure read 8 counts vs true 32 - the expected finding: the system hears four cycles of eight with no signal they form one longer phrase. Distinct from clips 5-8s sparse-marker undercount - every count was spoken cleanly here; this is a pure phrase-boundary/grouping miss.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="43" customHeight="1">
       <c r="A24" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 19 (both sides, 32-count, 4/4) — sides right, counts wrong
Metronome 104 confirmed, 32 counts, "other side" spoken between rounds,
32 counts again (numbering resets, not 33-64).

Tempo (0.1% err) and meter both correct. Sides correctly read 2 — the
verbal "other side" cue worked as a grouping signal. Counts read 8, not
32 — the same phrase-boundary miss as clip 18. Interesting split on the
same underlying audio shape: side-detection succeeded where
phrase-length grouping failed.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1856,7 +1856,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="43" customHeight="1">
+    <row r="24" ht="90" customHeight="1">
       <c r="A24" s="4" t="n">
         <v>19</v>
       </c>
@@ -1902,10 +1902,22 @@
           <t>Same 32-count idea as clip 18: count it through once, say "other side", and count it through again. Sides = both, counts stay 32 (one side's phrase — sides are never multiplied into counts).</t>
         </is>
       </c>
-      <c r="L24" s="6" t="inlineStr"/>
-      <c r="M24" s="6" t="inlineStr"/>
-      <c r="N24" s="6" t="inlineStr"/>
-      <c r="O24" s="7" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N24" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="O24" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. 32 counts, "other side" spoken between rounds, 32 counts again (numbering resets). Pipeline: tempo 104.1 (0.1% err) and meter 4/4 both correct. Sides correctly read 2 - the other side cue worked. Counts read 8 vs true 32 - same phrase-boundary miss as clip 18. Interesting split: side-detection succeeded where phrase-length grouping failed on the same underlying shape.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="43" customHeight="1">
       <c r="A25" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 20 (waltz lilt, 3/4 @88) — near-miss on the arbitration gate
Metronome 88 confirmed, step names with downbeat lilt ("DOWN two three,
LIFT two three"), one word per click (no subdivision), 8 counts.

Tempo correct (4.1% err). Meter read 4/4 duple instead of 3/4 none —
another waltz-precedence instance (clips 6, 13). Notably close this
time: the marker path read 90.6 BPM at 59% confidence with 24 beats —
one point under ADR-013's 60% arbitration-gate threshold. Had it
cleared, the correct in-band marker reading would have won instead of
the onset path. Counts read 24 vs true 8.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1919,7 +1919,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="43" customHeight="1">
+    <row r="25" ht="105" customHeight="1">
       <c r="A25" s="4" t="n">
         <v>20</v>
       </c>
@@ -1969,10 +1969,22 @@
           <t>A waltz with real LILT — let your voice swing the downbeat ("DOWN two three, LIFT two three…"), balancé feel, metronome 88. 8 or 16 counts (write which in 'Actual counts'), two or three times through.</t>
         </is>
       </c>
-      <c r="L25" s="6" t="inlineStr"/>
-      <c r="M25" s="6" t="inlineStr"/>
-      <c r="N25" s="6" t="inlineStr"/>
-      <c r="O25" s="7" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M25" s="6" t="n">
+        <v>88</v>
+      </c>
+      <c r="N25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O25" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. Step names, downbeat lilt (DOWN two three, LIFT two three), one word per click no subdivision, 8 counts. Pipeline: tempo 91.6 (4.1% err) - GREEN. Meter read 4/4 duple vs true 3/4 none - another waltz-precedence instance (clips 6, 13). Near-miss: marker path read 90.6 BPM at 59% confidence - one point under ADR-013s 60% arbitration gate. Had it cleared, the correct in-band marker reading would have won. Counts 24 vs true 8.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="43" customHeight="1">
       <c r="A26" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 21 (grand allegro, 4/4 @96) — real tempo drift, not detection
Metronome 96 confirmed, big/sharp full-voice accents on the jumps
("grand jete, and assemble... up two three down two three... jump jump
and jump"), 32 counts.

Tempo read 115.1 BPM, a 19.9% miss — not a clean x2/x3 metric-level
ratio, and the first onset section is nearly perfectly steady (CV=0.00)
at that faster tempo. Reads as genuine tempo drift (energetic delivery
rushing ahead of the click) rather than a detection artifact — a
plausible pedagogical phenomenon the onset detector has no way to
distinguish from "the metronome actually was faster." Counts abstained,
consistent with clips 9/14/17's pattern of declining rather than
committing when the marker stream is irregular.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -1986,7 +1986,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="43" customHeight="1">
+    <row r="26" ht="105" customHeight="1">
       <c r="A26" s="4" t="n">
         <v>21</v>
       </c>
@@ -2032,10 +2032,22 @@
           <t>Grand-allegro energy: big, sharp, accented marking — "and GRAND jeté, and RUN run RUN, and assemblé…" — full voice, 8 to 16 counts. Note the length in 'Actual counts'.</t>
         </is>
       </c>
-      <c r="L26" s="6" t="inlineStr"/>
-      <c r="M26" s="6" t="inlineStr"/>
-      <c r="N26" s="6" t="inlineStr"/>
-      <c r="O26" s="7" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M26" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="N26" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="O26" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. Grand-allegro energy, big full-voice accents on jumps, 32 counts, mixed step-name bursts and counted numbers. Pipeline: tempo 115.1 (19.9% err) - RED, not a clean x2/x3 metric-level ratio, first section nearly perfectly steady (CV=0.00) at that faster tempo - reads as real tempo drift (energy/excitement rushing ahead of click), not a detection artifact. Meter follows the wrong tempo. Counts abstained - phrase mixes styles rather than one uniform pattern.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="56" customHeight="1">
       <c r="A27" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 22 (mixed quantities, 4/4 @104) — the trap works as designed
Metronome 104 confirmed, numbers used only as quantities inside natural
step-name phrasing ("we take two tendus to the front, then one to the
back, three quick chatés...") never as actual beat counts, true phrase
32 counts.

The trap worked exactly as designed: Gemini found zero beat markers —
no coherent classification, since none of the spoken numbers line up
with the real count. The onset detector, with nothing else to go on,
locked onto irregular word-to-word spacing and read 170 BPM (halved to
85 by the band snap), an 18.3% miss. Counts correctly abstained rather
than guessing. Also reported 2 sides despite no "other side" cue
anywhere in the transcript — an artifact, left unscored.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -2049,7 +2049,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="56" customHeight="1">
+    <row r="27" ht="105" customHeight="1">
       <c r="A27" s="4" t="n">
         <v>22</v>
       </c>
@@ -2099,10 +2099,22 @@
           <t>The trap clip. Mark with step names but use numbers as AMOUNTS, never as counts: "we take TWO tendus front, ONE more, and THREE quick ones to the side…". Speak in tempo. The numbers must not line up with the count — that's what fools machines. Write the TRUE phrase length in 'Actual counts'.</t>
         </is>
       </c>
-      <c r="L27" s="6" t="inlineStr"/>
-      <c r="M27" s="6" t="inlineStr"/>
-      <c r="N27" s="6" t="inlineStr"/>
-      <c r="O27" s="7" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N27" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="O27" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. The trap clip - numbers used only as quantities in natural step-name phrasing (we take two tendus front, then one to the back, three quick chates...), never as beat counts, true phrase 32 counts. Trap worked exactly as designed: Gemini found ZERO beat markers. Onset detector locked onto irregular word spacing, read 170 (halved to 85 by band-snap) - 18.3% miss. Counts correctly abstained. Also reported 2 sides though no other side cue exists - likely an artifact, not scored.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 23 (quiet/mumbled, 4/4 @100) — wholesale word loss
Metronome 100 confirmed, end-of-day quiet/low-energy/mumbled marking,
16 counts. Bounce filename saved truncated in the source folder
("g-names-4-4-100-quiet.mp3"), corrected on copy into the repo.

Whisper's transcript is only 12 tokens for the whole clip — "reverence,
and then we close, and reverence, and now we're done, yeah" — far short
of a 16-count phrase. Reads as wholesale word loss from the quiet
delivery, distinct from clips 5-8's deliberate silent-count pattern.
Gemini found only 3 usable beats at 48% confidence. Tempo (19.3% err),
meter, and counts (8 vs true 16, roughly half the phrase) all wrong.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -2116,7 +2116,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="30" customHeight="1">
+    <row r="28" ht="105" customHeight="1">
       <c r="A28" s="4" t="n">
         <v>23</v>
       </c>
@@ -2162,10 +2162,22 @@
           <t>End-of-day voice: quiet, low-energy, slightly mumbled marking of any simple exercise — still in tempo with the earbud. 8 counts, twice through.</t>
         </is>
       </c>
-      <c r="L28" s="6" t="inlineStr"/>
-      <c r="M28" s="6" t="inlineStr"/>
-      <c r="N28" s="6" t="inlineStr"/>
-      <c r="O28" s="7" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M28" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N28" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O28" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. End-of-day quiet/mumbled voice, 16 counts (bounce saved with truncated filename g-names-4-4-100-quiet.mp3, corrected on copy). Whisper transcript is only 12 tokens total (reverence, and then we close, and reverence, and now were done, yeah) - wholesale word loss from the quiet delivery, not just occasional gaps. Gemini found only 3 beats at 48% conf. Pipeline: tempo 119.3 (19.3% err), meter 4/4 duple, counts 8 vs true 16 - all RED, roughly half the phrase lost.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="43" customHeight="1">
       <c r="A29" s="4" t="n">

</xml_diff>

<commit_message>
feat: rig clip 24 (free coda, 4/4 @104) — final clip, phrase boundary caught
Metronome 104 confirmed, 32-count phrase followed by a genuinely free,
out-of-tempo coda ("the other way... and balance... and stop") with
irregular pauses. Bounce saved with a trailing space in the filename,
corrected on copy. Last clip on the capture checklist — all 24 done.

Interesting partial success: the onset detector's rhythmic-section
boundary (2.3-20.8s) lines up almost exactly with the true 32-count
phrase length at 104 BPM, correctly excluding the free coda — exactly
the boundary this clip was designed to test. But tempo within that
correctly-bounded section still read low (72.2, 30.6% miss, CV=0.01):
natural descriptive step-name phrasing doesn't put one word on every
click the way strict counting does. Counts abstained.
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -2179,7 +2179,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="43" customHeight="1">
+    <row r="29" ht="120" customHeight="1">
       <c r="A29" s="4" t="n">
         <v>24</v>
       </c>
@@ -2225,10 +2225,22 @@
           <t>Mark a 32-count phrase, then finish FREELY with "aaand port de bras… and balance…" as an ending outside the count. 'Counts per phrase' stays 32 — the ending is NOT included (whether the machine knows that is the test).</t>
         </is>
       </c>
-      <c r="L29" s="6" t="inlineStr"/>
-      <c r="M29" s="6" t="inlineStr"/>
-      <c r="N29" s="6" t="inlineStr"/>
-      <c r="O29" s="7" t="inlineStr"/>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>104</v>
+      </c>
+      <c r="N29" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08. 32-count phrase (turning around and then we drop... jump jump jump port de bras) then genuinely free out-of-tempo coda (the other way, and balance, and stop) with irregular pauses. Interesting partial success: onset section boundary (2.3-20.8s) lines up almost exactly with the true 32-count phrase length at 104bpm - correctly excluded the free coda. But tempo within that section still read low (72.2, 30.6% miss, CV=0.01) - descriptive phrasing doesnt put one word per click. Counts abstained. Final clip on the sheet - all 24 done.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
feat: ADR-015 accepted — owner override of the tripped kill criterion, on the record
The gate fired as designed and the override is documented, not laundered:
plies-demo's lost green was fake (eight sections spanning 59.5-262.8 BPM
= no measurement existed); waltz-lilt is a genuine, documented trade
(interval data cannot split stretched-beat from two-beats); the
explained.counts abstained->wrong flip the totals hid is named; clips
21/23 luck-flagged in their case notes against future flip-back panic.
Prediction scorecard recorded honestly: 1/3 pre-registered flips landed.
Gate amendment: typed gates — zero-regression stays for logic changes,
diagnosed-regression gate (net metric + ECE improvement, zero
UNdiagnosed regressions, knife-edge rows can't gate at n=29) for
measurement changes. ECE 0.401->0.291.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evals/capture-checklist.xlsx
+++ b/docs/evals/capture-checklist.xlsx
@@ -869,7 +869,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1">
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
@@ -932,7 +932,7 @@
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-07, take 2 (take 1 bounced silent). FIRST 6/8 recognized — accents worked. Onset tempo dragged to 84.7 by agogic bar-boundary gaps (spoke 96.3 on the 100 click); tempo row honestly red. Markers 96.3@51% under gate again.</t>
+          <t>2026-08-07, take 2 (take 1 bounced silent). FIRST 6/8 recognized — accents worked. Onset tempo dragged to 84.7 by agogic bar-boundary gaps (spoke 96.3 on the 100 click); tempo row honestly red. Markers 96.3@51% under gate again. ADR-015: tempo flipped GREEN (grid-fit rescued the agogic read) — meter triple with it.</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="O25" s="7" t="inlineStr">
         <is>
-          <t>2026-08-08. Step names, downbeat lilt (DOWN two three, LIFT two three), one word per click no subdivision, 8 counts. Pipeline: tempo 91.6 (4.1% err) - GREEN. Meter read 4/4 duple vs true 3/4 none - another waltz-precedence instance (clips 6, 13). Near-miss: marker path read 90.6 BPM at 59% confidence - one point under ADR-013s 60% arbitration gate. Had it cleared, the correct in-band marker reading would have won. Counts 24 vs true 8.</t>
+          <t>2026-08-08. Step names, downbeat lilt (DOWN two three, LIFT two three), one word per click no subdivision, 8 counts. Pipeline: tempo 91.6 (4.1% err) - GREEN. Meter read 4/4 duple vs true 3/4 none - another waltz-precedence instance (clips 6, 13). Near-miss: marker path read 90.6 BPM at 59% confidence - one point under ADR-013s 60% arbitration gate. Had it cleared, the correct in-band marker reading would have won. Counts 24 vs true 8. ADR-015: tempo went red — genuinely ambiguous gaps (stretched beat vs two beats); the documented trade.</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="O26" s="7" t="inlineStr">
         <is>
-          <t>2026-08-08. Grand-allegro energy, big full-voice accents on jumps, 32 counts, mixed step-name bursts and counted numbers. Pipeline: tempo 115.1 (19.9% err) - RED, not a clean x2/x3 metric-level ratio, first section nearly perfectly steady (CV=0.00) at that faster tempo - reads as real tempo drift (energy/excitement rushing ahead of click), not a detection artifact. Meter follows the wrong tempo. Counts abstained - phrase mixes styles rather than one uniform pattern.</t>
+          <t>2026-08-08. Grand-allegro energy, big full-voice accents on jumps, 32 counts, mixed step-name bursts and counted numbers. Pipeline: tempo 115.1 (19.9% err) - RED, not a clean x2/x3 metric-level ratio, first section nearly perfectly steady (CV=0.00) at that faster tempo - reads as real tempo drift (energy/excitement rushing ahead of click), not a detection artifact. Meter follows the wrong tempo. Counts abstained - phrase mixes styles rather than one uniform pattern. ADR-015: flipped green by LUCK (words still lost); expect flip-back when ASR improves.</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-08. End-of-day quiet/mumbled voice, 16 counts (bounce saved with truncated filename g-names-4-4-100-quiet.mp3, corrected on copy). Whisper transcript is only 12 tokens total (reverence, and then we close, and reverence, and now were done, yeah) - wholesale word loss from the quiet delivery, not just occasional gaps. Gemini found only 3 beats at 48% conf. Pipeline: tempo 119.3 (19.3% err), meter 4/4 duple, counts 8 vs true 16 - all RED, roughly half the phrase lost.</t>
+          <t>2026-08-08. End-of-day quiet/mumbled voice, 16 counts (bounce saved with truncated filename g-names-4-4-100-quiet.mp3, corrected on copy). Whisper transcript is only 12 tokens total (reverence, and then we close, and reverence, and now were done, yeah) - wholesale word loss from the quiet delivery, not just occasional gaps. Gemini found only 3 beats at 48% conf. Pipeline: tempo 119.3 (19.3% err), meter 4/4 duple, counts 8 vs true 16 - all RED, roughly half the phrase lost. ADR-015: flipped green by LUCK (words still lost); expect flip-back when ASR improves.</t>
         </is>
       </c>
     </row>

</xml_diff>